<commit_message>
Update Summer break calendar1.xlsx
</commit_message>
<xml_diff>
--- a/Summer break calendar1.xlsx
+++ b/Summer break calendar1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexc\OneDrive\Documents\NewGame+\NewGame-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{017CC16F-B261-493D-B10E-1DD7AB374308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B4277E9-6169-430D-8029-ADEABDB270FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="43470" yWindow="2100" windowWidth="19200" windowHeight="9975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38265" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summer holiday" sheetId="13" r:id="rId1"/>
@@ -64,9 +64,6 @@
   </si>
   <si>
     <t>Start Sentinel enemy</t>
-  </si>
-  <si>
-    <t>Finish level 4, start CynTessa</t>
   </si>
   <si>
     <t>Finish CynTessa, start Level 5</t>
@@ -209,6 +206,27 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t>Finish level 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, start CynTessa</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Finish Sentinels</t>
     </r>
     <r>
@@ -218,7 +236,26 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">, Start level 4, </t>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Start level 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Avenir Next LT Pro"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
     </r>
     <r>
       <rPr>
@@ -1014,6 +1051,12 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="9" applyFont="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="9" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="9" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1022,12 +1065,6 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="15" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="9" applyFont="1" applyBorder="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="9" applyFont="1" applyBorder="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="17">
@@ -40554,45 +40591,45 @@
     <row r="2" spans="1:16" s="3" customFormat="1" ht="80.150000000000006" customHeight="1" x14ac:dyDescent="1.85">
       <c r="A2" s="2"/>
       <c r="B2" s="40"/>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
       <c r="J2" s="2"/>
       <c r="K2" s="4"/>
-      <c r="L2" s="47" t="s">
+      <c r="L2" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="47"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="47"/>
-      <c r="P2" s="47"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="49"/>
     </row>
     <row r="3" spans="1:16" ht="50.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="41"/>
-      <c r="C3" s="49">
+      <c r="C3" s="51">
         <f ca="1">IF(MONTH(TODAY())&gt;9,YEAR(TODAY())+1,YEAR(TODAY()))</f>
         <v>2025</v>
       </c>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="49"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
       <c r="J3" s="6"/>
       <c r="K3" s="5"/>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="47"/>
-      <c r="O3" s="47"/>
-      <c r="P3" s="47"/>
+      <c r="L3" s="49"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="49"/>
+      <c r="O3" s="49"/>
+      <c r="P3" s="49"/>
     </row>
     <row r="4" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
@@ -40967,22 +41004,22 @@
       <c r="B18" s="41"/>
       <c r="C18" s="27"/>
       <c r="D18" s="45" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E18" s="46" t="s">
         <v>3</v>
       </c>
       <c r="F18" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="31" t="s">
+      <c r="H18" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="27" t="s">
-        <v>19</v>
-      </c>
       <c r="I18" s="27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J18" s="6"/>
       <c r="K18" s="5"/>
@@ -41034,10 +41071,10 @@
       <c r="E20" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="F20" s="50" t="s">
+      <c r="F20" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="G20" s="51" t="s">
+      <c r="G20" s="48" t="s">
         <v>7</v>
       </c>
       <c r="H20" s="27" t="s">
@@ -41089,19 +41126,19 @@
       <c r="B22" s="41"/>
       <c r="C22" s="27"/>
       <c r="D22" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="E22" s="27" t="s">
+      <c r="F22" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="F22" s="24" t="s">
+      <c r="G22" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G22" s="31" t="s">
-        <v>11</v>
-      </c>
       <c r="H22" s="27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I22" s="27"/>
       <c r="J22" s="6"/>
@@ -41149,10 +41186,10 @@
       <c r="B24" s="41"/>
       <c r="C24" s="27"/>
       <c r="D24" s="27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F24" s="27"/>
       <c r="G24" s="27"/>
@@ -41540,6 +41577,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -41557,15 +41603,6 @@
     <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -41881,6 +41918,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD7FBEAE-5747-42F6-91A2-F7FF653B21B7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97A5FD82-1F22-49EA-9704-A6D55C618F6D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -41888,14 +41933,6 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
     <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
     <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD7FBEAE-5747-42F6-91A2-F7FF653B21B7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>